<commit_message>
build screens and api
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-62_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-62_Test_Cases.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1354,8 +1354,38 @@
       </c>
       <c r="F33" s="9" t="n"/>
     </row>
+    <row r="35" ht="206.5" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Code reviewed</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>src/app/events/[id]/update/page.tsx
+src/app/events/[id]/page.tsx
+src/app/events/[id]/equipment/page.tsx
+src/app/api/events/[id]/information/route.ts
+src/app/api/events/[id]/equipment/route.ts
+src/app/api/events/[id]/equipment/[requestId]/route.ts
+src/lib/eventChangeImpact.ts
+src/lib/applyEventInformation.ts
+src/lib/eventInformationForm.ts
+src/lib/beginPlanning.ts
+src/lib/permissions.ts
+src/lib/validation/events.ts
+prisma/schema.prisma
+prisma/migrations/20261005120000_add_event_change_review_flags/migration.sql
+scripts/seed-spm62.ts</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E30:F30"/>
@@ -1373,6 +1403,7 @@
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="E31:F31"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -3093,13 +3124,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="58" customHeight="1">
+    <row r="2" ht="71.5" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written before the code (TDD, 2026-10-05). Every label, message, page address and rule below marked DECIDED was chosen here, in the style of the existing screens, and is what the developer now builds to. Change any of them before the code is written and update the cases with it.</t>
+          <t>Written before the code (TDD, 2026-10-05), then checked against the built screens the same day: every label, message and page address in the cases is what the code shows. Entries marked DECIDED were chosen by the team rather than taken from the story; change them in code and cases together.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
@@ -3170,13 +3201,13 @@
       </c>
       <c r="C8" s="11" t="n"/>
     </row>
-    <row r="9" ht="355" customHeight="1">
+    <row r="9" ht="395.5" customHeight="1">
       <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Fixture events, to build as `scripts/seed-spm62.ts` (`npm run fixtures:spm62`) and to append to prisma/seed.ts once the review-flag columns exist. All are coordinated by Daniel Tan, and each has a unique title. (1) 'SPM62 Harbour Leadership Summit': Planning, organiser Evelyn Chen, 17 Mar 2027 09:00–17:00, attendance 80, layout theatre, required 'Fixed ceiling projector', Approved booking Orchard Seminar Room (ORC-SEM), 4K Portable Projector × 2 Reserved, registration on with capacity 100, closing 10 Mar 2027 18:00, and 12 attendees registered. (2) 'SPM62 Kirana Supplier Day': Planning, organiser Faridah Aziz, 21 Apr 2027 10:00–16:00, attendance 60, Approved booking Changi Conference Centre (CBP-CONF), Handheld Wireless Mic × 4 Reserved, registration on with 8 registered. (3) 'SPM62 Bayu Energy Outlook': Approved, organiser Hakim Zulkifli, 12 May 2027 09:00–12:00, attendance 40, no arrangements, registration off. (4) 'SPM62 Anchorpoint Logistics Forum': Approved, organiser Melissa Yap, 18 May 2027 09:00–12:00, attendance 50, no arrangements. (5) 'SPM62 Straits Pharmacy Forum': Confirmed, organiser Evelyn Chen, 9 Jun 2027 09:00–17:00, attendance 120, Approved booking Marina Auditorium (MAR-AUD), Powered Speaker × 2 Reserved, registration on with capacity 150 and 20 registered. (6) 'SPM62 Meridian Quarterly Review': Confirmed, organiser James Koh, 16 Jun 2027 14:00–17:00, attendance 30, Approved booking Marina Boardroom 1 (MAR-BR1), registration off. (7) 'SPM62 Sundara Hospitality Showcase': Confirmed, organiser Dewi Kartika, 23 Jun 2027 10:00–18:00, attendance 70, Approved booking Orchard Gallery (ORC-GAL), no equipment. (8) 'SPM62 Civic Learning Day': Under review, organiser Grace Abdullah, 7 Jul 2027. (9) 'SPM62 Pearl Delta Plant Tour': Completed, organiser Samuel Ong, 10 Sep 2026.</t>
+          <t>Fixture events: `scripts/seed-spm62.ts` (`npm run fixtures:spm62`) creates them with their bookings, equipment, registrations and required facility; prisma/seed.ts creates the same events only (appended last), so run the script once after a full reseed. All are coordinated by Daniel Tan, and each has a unique title. (1) 'SPM62 Harbour Leadership Summit': Planning, organiser Evelyn Chen, 17 Mar 2027 09:00–17:00, attendance 80, layout theatre, required 'Fixed ceiling projector', Approved booking Orchard Seminar Room (ORC-SEM), 4K Portable Projector × 2 Reserved, registration on with capacity 100, closing 15 Mar 2027 09:00 (two days before, as every seeded event's registration does), and 12 attendees registered. (2) 'SPM62 Kirana Supplier Day': Planning, organiser Faridah Aziz, 21 Apr 2027 10:00–16:00, attendance 60, Approved booking Changi Conference Centre (CBP-CONF), Handheld Wireless Mic × 4 Reserved, registration on with 8 registered. (3) 'SPM62 Bayu Energy Outlook': Approved, organiser Hakim Zulkifli, 12 May 2027 09:00–12:00, attendance 40, no arrangements, registration off. (4) 'SPM62 Anchorpoint Logistics Forum': Approved, organiser Melissa Yap, 18 May 2027 09:00–12:00, attendance 50, no arrangements. (5) 'SPM62 Straits Pharmacy Forum': Confirmed, organiser Evelyn Chen, 9 Jun 2027 09:00–17:00, attendance 120, Approved booking Marina Auditorium (MAR-AUD), Powered Speaker × 2 Reserved, registration on with capacity 150 and 20 registered. (6) 'SPM62 Meridian Quarterly Review': Confirmed, organiser James Koh, 16 Jun 2027 14:00–17:00, attendance 30, Approved booking Marina Boardroom 1 (MAR-BR1), registration off. (7) 'SPM62 Sundara Hospitality Showcase': Confirmed, organiser Dewi Kartika, 23 Jun 2027 10:00–18:00, attendance 70, Approved booking Orchard Gallery (ORC-GAL), no equipment. (8) 'SPM62 Civic Learning Day': Under review, organiser Grace Abdullah, 7 Jul 2027. (9) 'SPM62 Pearl Delta Plant Tour': Completed, organiser Samuel Ong, 10 Sep 2026.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
@@ -3575,8 +3606,8 @@
         <is>
           <t>1. Click 'All Events' in the sidebar and open 'SPM62 Harbour Leadership Summit'
 2. Click 'Edit event information'
-3. Change 'Starts at' to 10 Mar 2027, 09:00
-4. Change 'Ends at' to 10 Mar 2027, 17:00
+3. Change 'Starts at' to 14 Mar 2027, 09:00
+4. Change 'Ends at' to 14 Mar 2027, 17:00
 5. Click 'Save changes'
 6. Click 'Cancel'</t>
         </is>
@@ -3590,7 +3621,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM62 Harbour Leadership Summit | Registration closes: 10 Mar 2027, 18:00 | Proposed: 10 Mar 2027, 09:00–17:00</t>
+          <t>Event: SPM62 Harbour Leadership Summit | Registration closes: 15 Mar 2027, 09:00 | Proposed: 14 Mar 2027, 09:00–17:00</t>
         </is>
       </c>
     </row>

</xml_diff>